<commit_message>
Update Projectplan status phase 1.4 & 2
</commit_message>
<xml_diff>
--- a/Documentation/project-plan.xlsx
+++ b/Documentation/project-plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ebiru\code\Informatik-2.Jahr\IPT6.1\IPT6.1-Productivity-Game\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanji\Documents\GitHub\IPT6.1-Productivity-Game\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEEB3465-5B43-4D6A-B68A-70F0F5621A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523EACA2-8543-4588-B2BE-7BA080DCC1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-3780" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Idea Planner" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,8 @@
   <definedNames>
     <definedName name="ColumnTitle1">Tasks[[#Headers],[ Task Status Indicator]]</definedName>
     <definedName name="ColumnTitleRegion1..G5.1">'Idea Planner'!$B$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Idea Planner'!$6:$6</definedName>
     <definedName name="PlanDueDate">'Idea Planner'!$E$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Idea Planner'!$6:$6</definedName>
     <definedName name="RowTitleRegion1..E3">'Idea Planner'!$D$2</definedName>
     <definedName name="RowTitleRegion2..G3">'Idea Planner'!$F$2</definedName>
   </definedNames>
@@ -840,26 +840,26 @@
     </xf>
   </cellXfs>
   <cellStyles count="20">
-    <cellStyle name="Calculation" xfId="16" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Berechnung" xfId="16" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Besuchter Hyperlink" xfId="6" builtinId="9" customBuiltin="1"/>
     <cellStyle name="Center aligned" xfId="9" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Comma" xfId="10" builtinId="3" customBuiltin="1"/>
-    <cellStyle name="Comma [0]" xfId="11" builtinId="6" customBuiltin="1"/>
-    <cellStyle name="Currency" xfId="12" builtinId="4" customBuiltin="1"/>
-    <cellStyle name="Currency [0]" xfId="13" builtinId="7" customBuiltin="1"/>
+    <cellStyle name="Dezimal [0]" xfId="11" builtinId="6" customBuiltin="1"/>
     <cellStyle name="Due Date" xfId="18" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Explanatory Text" xfId="7" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
-    <cellStyle name="Per cent" xfId="14" builtinId="5" customBuiltin="1"/>
+    <cellStyle name="Erklärender Text" xfId="7" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Komma" xfId="10" builtinId="3" customBuiltin="1"/>
+    <cellStyle name="Link" xfId="5" builtinId="8" customBuiltin="1"/>
     <cellStyle name="Plan Due Date" xfId="8" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Prozent" xfId="14" builtinId="5" customBuiltin="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0" customBuiltin="1"/>
     <cellStyle name="Status Icon Text" xfId="19" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
     <cellStyle name="Task Indicator" xfId="17" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Überschrift" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Überschrift 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Überschrift 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Überschrift 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Überschrift 4" xfId="15" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Währung" xfId="12" builtinId="4" customBuiltin="1"/>
+    <cellStyle name="Währung [0]" xfId="13" builtinId="7" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="11">
     <dxf>
@@ -1336,23 +1336,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:G133"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.54296875" customWidth="1"/>
+    <col min="1" max="1" width="2.5546875" customWidth="1"/>
     <col min="2" max="2" width="1" customWidth="1"/>
-    <col min="3" max="3" width="42.54296875" customWidth="1"/>
-    <col min="4" max="4" width="18.54296875" customWidth="1"/>
-    <col min="5" max="5" width="22.54296875" customWidth="1"/>
+    <col min="3" max="3" width="42.5546875" customWidth="1"/>
+    <col min="4" max="4" width="18.5546875" customWidth="1"/>
+    <col min="5" max="5" width="22.5546875" customWidth="1"/>
     <col min="6" max="6" width="31" customWidth="1"/>
-    <col min="7" max="7" width="43.453125" customWidth="1"/>
-    <col min="8" max="8" width="2.54296875" customWidth="1"/>
+    <col min="7" max="7" width="43.44140625" customWidth="1"/>
+    <col min="8" max="8" width="2.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
     </row>
-    <row r="2" spans="2:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
@@ -1366,7 +1366,7 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="2:7" ht="33" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:7" ht="33" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="34"/>
       <c r="C3" s="34"/>
       <c r="D3" s="10" t="s">
@@ -1382,7 +1382,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:7" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B4" s="35" t="s">
         <v>3</v>
       </c>
@@ -1394,7 +1394,7 @@
       <c r="F4" s="35"/>
       <c r="G4" s="35"/>
     </row>
-    <row r="5" spans="2:7" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:7" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="36" t="s">
         <v>145</v>
       </c>
@@ -1406,7 +1406,7 @@
       <c r="F5" s="36"/>
       <c r="G5" s="36"/>
     </row>
-    <row r="6" spans="2:7" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:7" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="8" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="G7" s="26"/>
     </row>
-    <row r="8" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1464,7 +1464,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1486,7 +1486,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1508,7 +1508,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1530,7 +1530,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="G12" s="28"/>
     </row>
-    <row r="13" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1568,7 +1568,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1590,7 +1590,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1612,7 +1612,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1634,7 +1634,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1656,7 +1656,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="G18" s="29"/>
     </row>
-    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1694,7 +1694,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1716,7 +1716,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1738,7 +1738,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1760,7 +1760,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1782,7 +1782,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1804,7 +1804,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1826,7 +1826,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1842,10 +1842,10 @@
       </c>
       <c r="G26" s="25"/>
     </row>
-    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C27" t="s">
         <v>22</v>
@@ -1854,17 +1854,17 @@
         <v>46093</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="F27" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" s="30" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>0</v>
@@ -1886,7 +1886,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="G29" s="25"/>
     </row>
-    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1924,7 +1924,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1940,10 +1940,10 @@
       </c>
       <c r="G31" s="17"/>
     </row>
-    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C32" t="s">
         <v>25</v>
@@ -1952,17 +1952,17 @@
         <v>46100</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>10</v>
+        <v>148</v>
       </c>
       <c r="F32" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="11" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -1984,7 +1984,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2006,7 +2006,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2028,7 +2028,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="G36" s="26"/>
     </row>
-    <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2066,7 +2066,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2088,7 +2088,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2110,7 +2110,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="G40" s="26"/>
     </row>
-    <row r="41" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2148,7 +2148,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="42" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2170,7 +2170,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2192,7 +2192,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2214,7 +2214,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2236,7 +2236,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="46" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2252,10 +2252,10 @@
       </c>
       <c r="G46" s="29"/>
     </row>
-    <row r="47" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C47" t="s">
         <v>43</v>
@@ -2264,20 +2264,20 @@
         <v>46107</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>10</v>
+        <v>148</v>
       </c>
       <c r="F47" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G47" s="27" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C48" t="s">
         <v>142</v>
@@ -2286,17 +2286,17 @@
         <v>46107</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>10</v>
+        <v>148</v>
       </c>
       <c r="F48" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G48" s="27" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2318,7 +2318,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2340,7 +2340,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2362,7 +2362,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="52" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2384,7 +2384,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="53" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2406,7 +2406,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="54" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2428,7 +2428,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="55" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2450,7 +2450,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="G56" s="29"/>
     </row>
-    <row r="57" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2488,7 +2488,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="58" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2510,7 +2510,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="59" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2532,7 +2532,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="60" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2554,7 +2554,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="61" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="G61" s="29"/>
     </row>
-    <row r="62" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2592,7 +2592,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="63" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2614,7 +2614,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="64" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2636,7 +2636,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="65" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="G65" s="29"/>
     </row>
-    <row r="66" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2674,7 +2674,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="67" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2696,7 +2696,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2718,7 +2718,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="69" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2740,7 +2740,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="70" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="G70" s="29"/>
     </row>
-    <row r="71" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2778,7 +2778,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="72" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2800,7 +2800,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="73" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2822,7 +2822,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="74" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2844,7 +2844,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="75" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2866,7 +2866,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="76" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="G76" s="29"/>
     </row>
-    <row r="77" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B77" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2904,7 +2904,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="78" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B78" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2926,7 +2926,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="79" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B79" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2948,7 +2948,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="80" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B80" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2970,7 +2970,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B81" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="G81" s="29"/>
     </row>
-    <row r="82" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B82" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3008,7 +3008,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="83" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B83" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3030,7 +3030,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="84" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B84" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3052,7 +3052,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="85" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B85" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3074,7 +3074,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="86" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B86" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="G86" s="29"/>
     </row>
-    <row r="87" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B87" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3112,7 +3112,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="88" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B88" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3134,7 +3134,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="89" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B89" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3156,7 +3156,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="90" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B90" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3178,7 +3178,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="91" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B91" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3200,7 +3200,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="92" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B92" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3222,7 +3222,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="93" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B93" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3238,7 +3238,7 @@
       </c>
       <c r="G93" s="29"/>
     </row>
-    <row r="94" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B94" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3260,7 +3260,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="95" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B95" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3282,7 +3282,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="96" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B96" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3304,7 +3304,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="97" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B97" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3326,7 +3326,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B98" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="G98" s="29"/>
     </row>
-    <row r="99" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B99" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3364,7 +3364,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="100" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B100" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3386,7 +3386,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="101" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B101" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3408,7 +3408,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="102" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B102" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3430,7 +3430,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="103" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B103" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="G103" s="29"/>
     </row>
-    <row r="104" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B104" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3468,7 +3468,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="105" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B105" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3490,7 +3490,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="106" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B106" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3512,7 +3512,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="107" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B107" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3534,7 +3534,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="108" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B108" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3550,7 +3550,7 @@
       </c>
       <c r="G108" s="29"/>
     </row>
-    <row r="109" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B109" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3572,7 +3572,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="110" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B110" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3594,7 +3594,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="111" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B111" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="G111" s="29"/>
     </row>
-    <row r="112" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B112" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3632,7 +3632,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="113" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B113" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3654,7 +3654,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="114" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B114" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3676,7 +3676,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="115" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B115" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3698,7 +3698,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="116" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B116" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="G116" s="29"/>
     </row>
-    <row r="117" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B117" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3736,7 +3736,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="118" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B118" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3758,7 +3758,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="119" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B119" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="G119" s="29"/>
     </row>
-    <row r="120" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B120" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3796,7 +3796,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="121" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B121" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3818,7 +3818,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="122" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B122" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3840,7 +3840,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="123" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B123" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3862,7 +3862,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="124" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B124" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="G124" s="29"/>
     </row>
-    <row r="125" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B125" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3900,7 +3900,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="126" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B126" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3922,7 +3922,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="127" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B127" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3944,7 +3944,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="128" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B128" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3966,7 +3966,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="129" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B129" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3988,7 +3988,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="130" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B130" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="G130" s="29"/>
     </row>
-    <row r="131" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B131" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -4026,7 +4026,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="132" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B132" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -4048,7 +4048,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="133" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B133" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>

</xml_diff>

<commit_message>
Delete User-Flow in Projectplan
</commit_message>
<xml_diff>
--- a/Documentation/project-plan.xlsx
+++ b/Documentation/project-plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanji\Documents\GitHub\IPT6.1-Productivity-Game\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523EACA2-8543-4588-B2BE-7BA080DCC1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EDFAFB-3A4A-4EC8-B1F8-54D3326967B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="148">
   <si>
     <t>Idea Planner</t>
   </si>
@@ -125,9 +125,6 @@
   </si>
   <si>
     <t>Zwecks- und Funktionsdefinition</t>
-  </si>
-  <si>
-    <t>Benutzerabläufe festlegen</t>
   </si>
   <si>
     <t>Wireframe-Tool auswählen</t>
@@ -1036,8 +1033,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tasks" displayName="Tasks" ref="B6:G133" totalsRowShown="0">
-  <autoFilter ref="B6:G133" xr:uid="{00000000-0009-0000-0100-000001000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tasks" displayName="Tasks" ref="B6:G132" totalsRowShown="0">
+  <autoFilter ref="B6:G132" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1335,7 +1332,7 @@
     <tabColor theme="4"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:G133"/>
+  <dimension ref="B1:G132"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.5546875" customWidth="1"/>
@@ -1396,12 +1393,12 @@
     </row>
     <row r="5" spans="2:7" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="36"/>
       <c r="D5" s="36"/>
       <c r="E5" s="36" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F5" s="36"/>
       <c r="G5" s="36"/>
@@ -1423,7 +1420,7 @@
         <v>9</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1432,7 +1429,7 @@
         <v/>
       </c>
       <c r="C7" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="16"/>
@@ -1454,14 +1451,14 @@
         <v>46063</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F8" s="9">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G8" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1476,14 +1473,14 @@
         <v>46063</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F9" s="9">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1498,14 +1495,14 @@
         <v>46063</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F10" s="9">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G10" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1514,20 +1511,20 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D11" s="7">
         <v>46063</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F11" s="9">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G11" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1536,7 +1533,7 @@
         <v/>
       </c>
       <c r="C12" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D12" s="19"/>
       <c r="E12" s="20"/>
@@ -1558,14 +1555,14 @@
         <v>46079</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F13" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G13" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1580,14 +1577,14 @@
         <v>46079</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F14" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G14" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1602,14 +1599,14 @@
         <v>46079</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F15" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G15" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1624,14 +1621,14 @@
         <v>46079</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F16" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G16" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1646,14 +1643,14 @@
         <v>46079</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F17" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G17" s="27" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1662,7 +1659,7 @@
         <v/>
       </c>
       <c r="C18" s="22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D18" s="23"/>
       <c r="E18" s="24"/>
@@ -1678,20 +1675,20 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D19" s="12">
         <v>46086</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F19" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G19" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1700,20 +1697,20 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D20" s="12">
         <v>46086</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F20" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1722,20 +1719,20 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D21" s="12">
         <v>46086</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F21" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G21" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1744,20 +1741,20 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D22" s="12">
         <v>46086</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F22" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G22" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1766,20 +1763,20 @@
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D23" s="12">
         <v>46086</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F23" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G23" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1788,20 +1785,20 @@
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D24" s="12">
         <v>46086</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F24" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G24" s="27" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1810,20 +1807,20 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D25" s="12">
         <v>46086</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F25" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G25" s="27" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1832,7 +1829,7 @@
         <v/>
       </c>
       <c r="C26" s="22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D26" s="23"/>
       <c r="E26" s="24"/>
@@ -1854,14 +1851,14 @@
         <v>46093</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F27" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G27" s="30" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1876,14 +1873,14 @@
         <v>46093</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F28" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>0</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1892,7 +1889,7 @@
         <v/>
       </c>
       <c r="C29" s="22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D29" s="23"/>
       <c r="E29" s="24"/>
@@ -1914,14 +1911,14 @@
         <v>46093</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F30" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>1</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1930,7 +1927,7 @@
         <v/>
       </c>
       <c r="C31" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D31" s="31"/>
       <c r="E31" s="32"/>
@@ -1943,7 +1940,7 @@
     <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C32" t="s">
         <v>25</v>
@@ -1952,20 +1949,20 @@
         <v>46100</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="F32" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C33" t="s">
         <v>26</v>
@@ -1974,75 +1971,75 @@
         <v>46100</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F33" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D34" s="12">
         <v>46100</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F34" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C35" t="s">
+      <c r="B35" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="D35" s="31"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="17" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G35" s="26"/>
+    </row>
+    <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C36" t="s">
         <v>27</v>
       </c>
-      <c r="D35" s="12">
-        <v>46100</v>
-      </c>
-      <c r="E35" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F35" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G35" s="11" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C36" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="D36" s="31"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="17" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G36" s="26"/>
+      <c r="D36" s="12">
+        <v>46107</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G36" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="11">
@@ -2063,7 +2060,7 @@
         <v>-1</v>
       </c>
       <c r="G37" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="38" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2085,46 +2082,46 @@
         <v>-1</v>
       </c>
       <c r="G38" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C39" t="s">
-        <v>30</v>
-      </c>
-      <c r="D39" s="12">
+      <c r="B39" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="D39" s="31"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="17" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G39" s="26"/>
+    </row>
+    <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>31</v>
+      </c>
+      <c r="D40" s="12">
         <v>46107</v>
       </c>
-      <c r="E39" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F39" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G39" s="27" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="D40" s="31"/>
-      <c r="E40" s="32"/>
-      <c r="F40" s="17" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G40" s="26"/>
+      <c r="E40" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G40" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="41" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="11">
@@ -2145,7 +2142,7 @@
         <v>-1</v>
       </c>
       <c r="G41" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="42" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2167,7 +2164,7 @@
         <v>-1</v>
       </c>
       <c r="G42" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2176,10 +2173,10 @@
         <v>-1</v>
       </c>
       <c r="C43" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D43" s="12">
-        <v>46107</v>
+        <v>46112</v>
       </c>
       <c r="E43" s="13" t="s">
         <v>10</v>
@@ -2189,7 +2186,7 @@
         <v>-1</v>
       </c>
       <c r="G43" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2198,7 +2195,7 @@
         <v>-1</v>
       </c>
       <c r="C44" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D44" s="12">
         <v>46112</v>
@@ -2211,46 +2208,46 @@
         <v>-1</v>
       </c>
       <c r="G44" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="45" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D45" s="12">
-        <v>46112</v>
-      </c>
-      <c r="E45" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F45" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G45" s="27" t="s">
-        <v>137</v>
-      </c>
+      <c r="B45" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C45" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="D45" s="23"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G45" s="29"/>
     </row>
     <row r="46" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C46" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="D46" s="23"/>
-      <c r="E46" s="24"/>
-      <c r="F46" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G46" s="29"/>
+      <c r="B46" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>0</v>
+      </c>
+      <c r="C46" t="s">
+        <v>42</v>
+      </c>
+      <c r="D46" s="12">
+        <v>46107</v>
+      </c>
+      <c r="E46" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="F46" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G46" s="27" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="47" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="11">
@@ -2258,42 +2255,42 @@
         <v>0</v>
       </c>
       <c r="C47" t="s">
-        <v>43</v>
+        <v>141</v>
       </c>
       <c r="D47" s="12">
         <v>46107</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F47" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
         <v>0</v>
       </c>
       <c r="G47" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="48" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="C48" t="s">
         <v>142</v>
       </c>
       <c r="D48" s="12">
-        <v>46107</v>
+        <v>46112</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>148</v>
+        <v>10</v>
       </c>
       <c r="F48" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G48" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="49" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2315,7 +2312,7 @@
         <v>-1</v>
       </c>
       <c r="G49" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="50" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2324,10 +2321,10 @@
         <v>-1</v>
       </c>
       <c r="C50" t="s">
-        <v>144</v>
+        <v>43</v>
       </c>
       <c r="D50" s="12">
-        <v>46112</v>
+        <v>46135</v>
       </c>
       <c r="E50" s="13" t="s">
         <v>10</v>
@@ -2337,7 +2334,7 @@
         <v>-1</v>
       </c>
       <c r="G50" s="27" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="51" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2359,7 +2356,7 @@
         <v>-1</v>
       </c>
       <c r="G51" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="52" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2381,7 +2378,7 @@
         <v>-1</v>
       </c>
       <c r="G52" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="53" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2403,7 +2400,7 @@
         <v>-1</v>
       </c>
       <c r="G53" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="54" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2415,7 +2412,7 @@
         <v>47</v>
       </c>
       <c r="D54" s="12">
-        <v>46135</v>
+        <v>46111</v>
       </c>
       <c r="E54" s="13" t="s">
         <v>10</v>
@@ -2425,46 +2422,46 @@
         <v>-1</v>
       </c>
       <c r="G54" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="55" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C55" t="s">
+      <c r="B55" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C55" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="D55" s="23"/>
+      <c r="E55" s="24"/>
+      <c r="F55" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G55" s="29"/>
+    </row>
+    <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B56" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C56" t="s">
         <v>48</v>
       </c>
-      <c r="D55" s="12">
+      <c r="D56" s="12">
         <v>46111</v>
       </c>
-      <c r="E55" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F55" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G55" s="27" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C56" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="D56" s="23"/>
-      <c r="E56" s="24"/>
-      <c r="F56" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G56" s="29"/>
+      <c r="E56" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G56" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="57" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="11">
@@ -2485,7 +2482,7 @@
         <v>-1</v>
       </c>
       <c r="G57" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="58" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2507,7 +2504,7 @@
         <v>-1</v>
       </c>
       <c r="G58" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="59" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2529,46 +2526,46 @@
         <v>-1</v>
       </c>
       <c r="G59" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="60" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C60" t="s">
+      <c r="B60" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C60" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="D60" s="23"/>
+      <c r="E60" s="24"/>
+      <c r="F60" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G60" s="29"/>
+    </row>
+    <row r="61" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C61" t="s">
         <v>52</v>
       </c>
-      <c r="D60" s="12">
+      <c r="D61" s="12">
         <v>46111</v>
       </c>
-      <c r="E60" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F60" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G60" s="27" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="61" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C61" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="D61" s="23"/>
-      <c r="E61" s="24"/>
-      <c r="F61" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G61" s="29"/>
+      <c r="E61" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F61" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G61" s="27" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="62" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="11">
@@ -2589,7 +2586,7 @@
         <v>-1</v>
       </c>
       <c r="G62" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="63" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2611,46 +2608,46 @@
         <v>-1</v>
       </c>
       <c r="G63" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="64" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C64" t="s">
+      <c r="B64" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C64" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="D64" s="23"/>
+      <c r="E64" s="24"/>
+      <c r="F64" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G64" s="29"/>
+    </row>
+    <row r="65" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B65" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C65" t="s">
         <v>55</v>
       </c>
-      <c r="D64" s="12">
-        <v>46111</v>
-      </c>
-      <c r="E64" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F64" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G64" s="27" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="65" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C65" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="D65" s="23"/>
-      <c r="E65" s="24"/>
-      <c r="F65" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G65" s="29"/>
+      <c r="D65" s="12">
+        <v>46114</v>
+      </c>
+      <c r="E65" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F65" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G65" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="66" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="11">
@@ -2671,7 +2668,7 @@
         <v>-1</v>
       </c>
       <c r="G66" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="67" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2693,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="G67" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="68" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2702,7 +2699,7 @@
         <v>-1</v>
       </c>
       <c r="C68" t="s">
-        <v>58</v>
+        <v>146</v>
       </c>
       <c r="D68" s="12">
         <v>46114</v>
@@ -2715,46 +2712,46 @@
         <v>-1</v>
       </c>
       <c r="G68" s="27" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="69" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C69" t="s">
-        <v>147</v>
-      </c>
-      <c r="D69" s="12">
+      <c r="B69" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C69" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="D69" s="23"/>
+      <c r="E69" s="24"/>
+      <c r="F69" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G69" s="29"/>
+    </row>
+    <row r="70" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B70" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>58</v>
+      </c>
+      <c r="D70" s="12">
         <v>46114</v>
       </c>
-      <c r="E69" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F69" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G69" s="27" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="70" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C70" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="D70" s="23"/>
-      <c r="E70" s="24"/>
-      <c r="F70" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G70" s="29"/>
+      <c r="E70" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F70" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G70" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="71" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="11">
@@ -2775,7 +2772,7 @@
         <v>-1</v>
       </c>
       <c r="G71" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="72" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2797,7 +2794,7 @@
         <v>-1</v>
       </c>
       <c r="G72" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="73" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2819,7 +2816,7 @@
         <v>-1</v>
       </c>
       <c r="G73" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="74" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2841,46 +2838,46 @@
         <v>-1</v>
       </c>
       <c r="G74" s="27" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="75" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C75" t="s">
+      <c r="B75" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C75" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="D75" s="23"/>
+      <c r="E75" s="24"/>
+      <c r="F75" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G75" s="29"/>
+    </row>
+    <row r="76" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B76" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C76" t="s">
         <v>63</v>
       </c>
-      <c r="D75" s="12">
-        <v>46114</v>
-      </c>
-      <c r="E75" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F75" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G75" s="27" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="76" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C76" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="D76" s="23"/>
-      <c r="E76" s="24"/>
-      <c r="F76" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G76" s="29"/>
+      <c r="D76" s="12">
+        <v>46116</v>
+      </c>
+      <c r="E76" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F76" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G76" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="77" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B77" s="11">
@@ -2901,7 +2898,7 @@
         <v>-1</v>
       </c>
       <c r="G77" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="78" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2923,7 +2920,7 @@
         <v>-1</v>
       </c>
       <c r="G78" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="79" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2945,46 +2942,46 @@
         <v>-1</v>
       </c>
       <c r="G79" s="27" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="80" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B80" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C80" t="s">
+      <c r="B80" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C80" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="D80" s="23"/>
+      <c r="E80" s="24"/>
+      <c r="F80" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G80" s="29"/>
+    </row>
+    <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B81" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C81" t="s">
         <v>67</v>
       </c>
-      <c r="D80" s="12">
+      <c r="D81" s="12">
         <v>46116</v>
       </c>
-      <c r="E80" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F80" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G80" s="27" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B81" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C81" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="D81" s="23"/>
-      <c r="E81" s="24"/>
-      <c r="F81" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G81" s="29"/>
+      <c r="E81" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F81" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G81" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="82" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B82" s="11">
@@ -3005,7 +3002,7 @@
         <v>-1</v>
       </c>
       <c r="G82" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="83" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3027,7 +3024,7 @@
         <v>-1</v>
       </c>
       <c r="G83" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="84" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3049,46 +3046,46 @@
         <v>-1</v>
       </c>
       <c r="G84" s="27" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="85" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B85" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C85" t="s">
+      <c r="B85" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C85" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="D85" s="12">
-        <v>46116</v>
-      </c>
-      <c r="E85" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F85" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G85" s="27" t="s">
-        <v>137</v>
-      </c>
+      <c r="D85" s="23"/>
+      <c r="E85" s="24"/>
+      <c r="F85" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G85" s="29"/>
     </row>
     <row r="86" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B86" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C86" s="22" t="s">
+      <c r="B86" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C86" t="s">
         <v>72</v>
       </c>
-      <c r="D86" s="23"/>
-      <c r="E86" s="24"/>
-      <c r="F86" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G86" s="29"/>
+      <c r="D86" s="12">
+        <v>46117</v>
+      </c>
+      <c r="E86" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F86" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G86" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="87" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B87" s="11">
@@ -3099,7 +3096,7 @@
         <v>73</v>
       </c>
       <c r="D87" s="12">
-        <v>46117</v>
+        <v>46119</v>
       </c>
       <c r="E87" s="13" t="s">
         <v>10</v>
@@ -3109,7 +3106,7 @@
         <v>-1</v>
       </c>
       <c r="G87" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="88" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3131,7 +3128,7 @@
         <v>-1</v>
       </c>
       <c r="G88" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="89" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3153,7 +3150,7 @@
         <v>-1</v>
       </c>
       <c r="G89" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="90" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3165,7 +3162,7 @@
         <v>76</v>
       </c>
       <c r="D90" s="12">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="E90" s="13" t="s">
         <v>10</v>
@@ -3175,7 +3172,7 @@
         <v>-1</v>
       </c>
       <c r="G90" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="91" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3197,46 +3194,46 @@
         <v>-1</v>
       </c>
       <c r="G91" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="92" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B92" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C92" t="s">
+      <c r="B92" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C92" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="D92" s="12">
-        <v>46120</v>
-      </c>
-      <c r="E92" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F92" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G92" s="27" t="s">
-        <v>137</v>
-      </c>
+      <c r="D92" s="23"/>
+      <c r="E92" s="24"/>
+      <c r="F92" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G92" s="29"/>
     </row>
     <row r="93" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B93" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C93" s="22" t="s">
+      <c r="B93" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C93" t="s">
         <v>79</v>
       </c>
-      <c r="D93" s="23"/>
-      <c r="E93" s="24"/>
-      <c r="F93" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G93" s="29"/>
+      <c r="D93" s="12">
+        <v>46123</v>
+      </c>
+      <c r="E93" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F93" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G93" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="94" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B94" s="11">
@@ -3257,7 +3254,7 @@
         <v>-1</v>
       </c>
       <c r="G94" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="95" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3279,7 +3276,7 @@
         <v>-1</v>
       </c>
       <c r="G95" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="96" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3301,46 +3298,46 @@
         <v>-1</v>
       </c>
       <c r="G96" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="97" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B97" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C97" t="s">
-        <v>83</v>
-      </c>
-      <c r="D97" s="12">
+      <c r="B97" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C97" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="D97" s="23"/>
+      <c r="E97" s="24"/>
+      <c r="F97" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G97" s="29"/>
+    </row>
+    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B98" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>99</v>
+      </c>
+      <c r="D98" s="12">
         <v>46123</v>
       </c>
-      <c r="E97" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F97" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G97" s="27" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B98" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C98" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="D98" s="23"/>
-      <c r="E98" s="24"/>
-      <c r="F98" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G98" s="29"/>
+      <c r="E98" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F98" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G98" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="99" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B99" s="11">
@@ -3351,7 +3348,7 @@
         <v>100</v>
       </c>
       <c r="D99" s="12">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="E99" s="13" t="s">
         <v>10</v>
@@ -3361,7 +3358,7 @@
         <v>-1</v>
       </c>
       <c r="G99" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="100" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3383,7 +3380,7 @@
         <v>-1</v>
       </c>
       <c r="G100" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="101" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3405,46 +3402,46 @@
         <v>-1</v>
       </c>
       <c r="G101" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="102" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B102" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C102" t="s">
+      <c r="B102" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C102" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="D102" s="12">
-        <v>46125</v>
-      </c>
-      <c r="E102" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F102" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G102" s="27" t="s">
-        <v>137</v>
-      </c>
+      <c r="D102" s="23"/>
+      <c r="E102" s="24"/>
+      <c r="F102" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G102" s="29"/>
     </row>
     <row r="103" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B103" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C103" s="22" t="s">
+      <c r="B103" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C103" t="s">
         <v>104</v>
       </c>
-      <c r="D103" s="23"/>
-      <c r="E103" s="24"/>
-      <c r="F103" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G103" s="29"/>
+      <c r="D103" s="12">
+        <v>46128</v>
+      </c>
+      <c r="E103" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F103" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G103" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="104" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B104" s="11">
@@ -3465,7 +3462,7 @@
         <v>-1</v>
       </c>
       <c r="G104" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="105" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3487,7 +3484,7 @@
         <v>-1</v>
       </c>
       <c r="G105" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="106" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3509,46 +3506,46 @@
         <v>-1</v>
       </c>
       <c r="G106" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="107" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B107" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C107" t="s">
+      <c r="B107" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C107" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="D107" s="12">
-        <v>46128</v>
-      </c>
-      <c r="E107" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F107" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G107" s="27" t="s">
-        <v>137</v>
-      </c>
+      <c r="D107" s="23"/>
+      <c r="E107" s="24"/>
+      <c r="F107" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G107" s="29"/>
     </row>
     <row r="108" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B108" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C108" s="22" t="s">
+      <c r="B108" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C108" t="s">
         <v>109</v>
       </c>
-      <c r="D108" s="23"/>
-      <c r="E108" s="24"/>
-      <c r="F108" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G108" s="29"/>
+      <c r="D108" s="12">
+        <v>46133</v>
+      </c>
+      <c r="E108" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F108" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G108" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="109" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B109" s="11">
@@ -3569,46 +3566,46 @@
         <v>-1</v>
       </c>
       <c r="G109" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="110" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B110" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C110" t="s">
+      <c r="B110" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C110" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="D110" s="12">
-        <v>46133</v>
-      </c>
-      <c r="E110" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F110" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G110" s="27" t="s">
-        <v>137</v>
-      </c>
+      <c r="D110" s="23"/>
+      <c r="E110" s="24"/>
+      <c r="F110" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G110" s="29"/>
     </row>
     <row r="111" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B111" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C111" s="22" t="s">
+      <c r="B111" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C111" t="s">
         <v>112</v>
       </c>
-      <c r="D111" s="23"/>
-      <c r="E111" s="24"/>
-      <c r="F111" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G111" s="29"/>
+      <c r="D111" s="12">
+        <v>46135</v>
+      </c>
+      <c r="E111" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F111" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G111" s="27" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="112" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B112" s="11">
@@ -3619,7 +3616,7 @@
         <v>113</v>
       </c>
       <c r="D112" s="12">
-        <v>46135</v>
+        <v>46142</v>
       </c>
       <c r="E112" s="13" t="s">
         <v>10</v>
@@ -3629,7 +3626,7 @@
         <v>-1</v>
       </c>
       <c r="G112" s="27" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="113" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3651,7 +3648,7 @@
         <v>-1</v>
       </c>
       <c r="G113" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="114" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3673,46 +3670,46 @@
         <v>-1</v>
       </c>
       <c r="G114" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="115" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B115" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C115" t="s">
+      <c r="B115" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C115" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="D115" s="12">
-        <v>46142</v>
-      </c>
-      <c r="E115" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F115" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G115" s="27" t="s">
-        <v>137</v>
-      </c>
+      <c r="D115" s="23"/>
+      <c r="E115" s="24"/>
+      <c r="F115" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G115" s="29"/>
     </row>
     <row r="116" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B116" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C116" s="22" t="s">
+      <c r="B116" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C116" t="s">
         <v>117</v>
       </c>
-      <c r="D116" s="23"/>
-      <c r="E116" s="24"/>
-      <c r="F116" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G116" s="29"/>
+      <c r="D116" s="12">
+        <v>46156</v>
+      </c>
+      <c r="E116" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F116" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G116" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="117" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B117" s="11">
@@ -3733,46 +3730,46 @@
         <v>-1</v>
       </c>
       <c r="G117" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="118" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B118" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C118" t="s">
+      <c r="B118" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C118" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="D118" s="12">
-        <v>46156</v>
-      </c>
-      <c r="E118" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F118" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G118" s="27" t="s">
-        <v>137</v>
-      </c>
+      <c r="D118" s="23"/>
+      <c r="E118" s="24"/>
+      <c r="F118" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G118" s="29"/>
     </row>
     <row r="119" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B119" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C119" s="22" t="s">
+      <c r="B119" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C119" t="s">
         <v>120</v>
       </c>
-      <c r="D119" s="23"/>
-      <c r="E119" s="24"/>
-      <c r="F119" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G119" s="29"/>
+      <c r="D119" s="12">
+        <v>46163</v>
+      </c>
+      <c r="E119" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F119" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G119" s="27" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="120" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B120" s="11">
@@ -3783,7 +3780,7 @@
         <v>121</v>
       </c>
       <c r="D120" s="12">
-        <v>46163</v>
+        <v>46170</v>
       </c>
       <c r="E120" s="13" t="s">
         <v>10</v>
@@ -3793,7 +3790,7 @@
         <v>-1</v>
       </c>
       <c r="G120" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="121" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3837,46 +3834,46 @@
         <v>-1</v>
       </c>
       <c r="G122" s="27" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="123" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B123" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C123" t="s">
+      <c r="B123" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C123" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="D123" s="12">
-        <v>46170</v>
-      </c>
-      <c r="E123" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F123" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G123" s="27" t="s">
-        <v>140</v>
-      </c>
+      <c r="D123" s="23"/>
+      <c r="E123" s="24"/>
+      <c r="F123" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G123" s="29"/>
     </row>
     <row r="124" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B124" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C124" s="22" t="s">
+      <c r="B124" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C124" t="s">
         <v>125</v>
       </c>
-      <c r="D124" s="23"/>
-      <c r="E124" s="24"/>
-      <c r="F124" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G124" s="29"/>
+      <c r="D124" s="12">
+        <v>46177</v>
+      </c>
+      <c r="E124" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F124" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G124" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="125" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B125" s="11">
@@ -3897,7 +3894,7 @@
         <v>-1</v>
       </c>
       <c r="G125" s="27" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="126" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3919,7 +3916,7 @@
         <v>-1</v>
       </c>
       <c r="G126" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="127" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3941,7 +3938,7 @@
         <v>-1</v>
       </c>
       <c r="G127" s="27" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="128" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3963,46 +3960,46 @@
         <v>-1</v>
       </c>
       <c r="G128" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="129" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B129" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C129" t="s">
+      <c r="B129" s="11" t="str">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v/>
+      </c>
+      <c r="C129" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="D129" s="12">
-        <v>46177</v>
-      </c>
-      <c r="E129" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F129" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G129" s="27" t="s">
-        <v>139</v>
-      </c>
+      <c r="D129" s="23"/>
+      <c r="E129" s="24"/>
+      <c r="F129" s="25" t="str">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v/>
+      </c>
+      <c r="G129" s="29"/>
     </row>
     <row r="130" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B130" s="11" t="str">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v/>
-      </c>
-      <c r="C130" s="22" t="s">
+      <c r="B130" s="11">
+        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
+        <v>-1</v>
+      </c>
+      <c r="C130" t="s">
         <v>131</v>
       </c>
-      <c r="D130" s="23"/>
-      <c r="E130" s="24"/>
-      <c r="F130" s="25" t="str">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v/>
-      </c>
-      <c r="G130" s="29"/>
+      <c r="D130" s="12">
+        <v>46185</v>
+      </c>
+      <c r="E130" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F130" s="11">
+        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
+        <v>-1</v>
+      </c>
+      <c r="G130" s="27" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="131" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B131" s="11">
@@ -4010,7 +4007,7 @@
         <v>-1</v>
       </c>
       <c r="C131" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="D131" s="12">
         <v>46185</v>
@@ -4023,7 +4020,7 @@
         <v>-1</v>
       </c>
       <c r="G131" s="27" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="132" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -4032,7 +4029,7 @@
         <v>-1</v>
       </c>
       <c r="C132" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="D132" s="12">
         <v>46185</v>
@@ -4045,29 +4042,7 @@
         <v>-1</v>
       </c>
       <c r="G132" s="27" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="133" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B133" s="11">
-        <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
-      </c>
-      <c r="C133" t="s">
-        <v>133</v>
-      </c>
-      <c r="D133" s="12">
-        <v>46185</v>
-      </c>
-      <c r="E133" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F133" s="11">
-        <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
-      </c>
-      <c r="G133" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -4079,7 +4054,7 @@
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B5:D5"/>
   </mergeCells>
-  <conditionalFormatting sqref="B7:B133">
+  <conditionalFormatting sqref="B7:B132">
     <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="num" val="-1"/>
@@ -4091,17 +4066,17 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F7:F133">
-    <cfRule type="expression" dxfId="5" priority="25">
+  <conditionalFormatting sqref="F7:F132">
+    <cfRule type="expression" dxfId="5" priority="31">
       <formula>F7=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="26">
+    <cfRule type="expression" dxfId="4" priority="32">
       <formula>F7=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="27">
+    <cfRule type="expression" dxfId="3" priority="33">
       <formula>F7=-1</formula>
     </cfRule>
-    <cfRule type="iconSet" priority="28">
+    <cfRule type="iconSet" priority="34">
       <iconSet iconSet="3Symbols2">
         <cfvo type="percent" val="0"/>
         <cfvo type="num" val="0"/>
@@ -4109,17 +4084,17 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G26:G35">
-    <cfRule type="expression" dxfId="2" priority="1">
+  <conditionalFormatting sqref="G26:G34">
+    <cfRule type="expression" dxfId="2" priority="39">
       <formula>G26=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="1" priority="40">
       <formula>G26=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="0" priority="41">
       <formula>G26=-1</formula>
     </cfRule>
-    <cfRule type="iconSet" priority="4">
+    <cfRule type="iconSet" priority="42">
       <iconSet iconSet="3Symbols2">
         <cfvo type="percent" val="0"/>
         <cfvo type="num" val="0"/>
@@ -4149,7 +4124,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:G1048576" xr:uid="{482F76EC-3095-4ECD-80A0-E3C86F6A9FD3}">
       <formula1>"Sanjivan,Egor,Sanjivan &amp; Egor, Unbestimmt"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Select an option from the list. Press Cancel then ALT+DOWN ARROW to open the drop-down list, then ENTER to make selection" sqref="E7:E133" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Select an option from the list. Press Cancel then ALT+DOWN ARROW to open the drop-down list, then ENTER to make selection" sqref="E7:E132" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Yes, No, Pending"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update projektplan phase 2
</commit_message>
<xml_diff>
--- a/Documentation/project-plan.xlsx
+++ b/Documentation/project-plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanji\Documents\GitHub\IPT6.1-Productivity-Game\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EDFAFB-3A4A-4EC8-B1F8-54D3326967B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B896466C-7B17-4091-8FEC-7C3A1E7898E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1984,7 +1984,7 @@
     <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C34" t="s">
         <v>140</v>
@@ -1993,11 +1993,11 @@
         <v>46100</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="F34" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" s="11" t="s">
         <v>138</v>
@@ -2022,7 +2022,7 @@
     <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C36" t="s">
         <v>27</v>
@@ -2031,11 +2031,11 @@
         <v>46107</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F36" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G36" s="27" t="s">
         <v>136</v>
@@ -2044,7 +2044,7 @@
     <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C37" t="s">
         <v>28</v>
@@ -2053,11 +2053,11 @@
         <v>46107</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F37" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G37" s="27" t="s">
         <v>136</v>

</xml_diff>

<commit_message>
Update Projectplan phase 2.2 & 2.3
</commit_message>
<xml_diff>
--- a/Documentation/project-plan.xlsx
+++ b/Documentation/project-plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanji\Documents\GitHub\IPT6.1-Productivity-Game\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B896466C-7B17-4091-8FEC-7C3A1E7898E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24884F2A-0C21-4041-B639-0A879839CBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Idea Planner" sheetId="1" r:id="rId1"/>
@@ -1333,23 +1333,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:G132"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.5546875" customWidth="1"/>
+    <col min="1" max="1" width="2.5703125" customWidth="1"/>
     <col min="2" max="2" width="1" customWidth="1"/>
-    <col min="3" max="3" width="42.5546875" customWidth="1"/>
-    <col min="4" max="4" width="18.5546875" customWidth="1"/>
-    <col min="5" max="5" width="22.5546875" customWidth="1"/>
+    <col min="3" max="3" width="42.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" customWidth="1"/>
+    <col min="5" max="5" width="22.5703125" customWidth="1"/>
     <col min="6" max="6" width="31" customWidth="1"/>
-    <col min="7" max="7" width="43.44140625" customWidth="1"/>
-    <col min="8" max="8" width="2.5546875" customWidth="1"/>
+    <col min="7" max="7" width="43.42578125" customWidth="1"/>
+    <col min="8" max="8" width="2.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
     </row>
-    <row r="2" spans="2:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
@@ -1363,7 +1363,7 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="2:7" ht="33" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:7" ht="33" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="34"/>
       <c r="C3" s="34"/>
       <c r="D3" s="10" t="s">
@@ -1379,7 +1379,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:7" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B4" s="35" t="s">
         <v>3</v>
       </c>
@@ -1391,7 +1391,7 @@
       <c r="F4" s="35"/>
       <c r="G4" s="35"/>
     </row>
-    <row r="5" spans="2:7" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="36" t="s">
         <v>144</v>
       </c>
@@ -1403,7 +1403,7 @@
       <c r="F5" s="36"/>
       <c r="G5" s="36"/>
     </row>
-    <row r="6" spans="2:7" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="G7" s="26"/>
     </row>
-    <row r="8" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1461,7 +1461,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1483,7 +1483,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1505,7 +1505,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1527,7 +1527,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="G12" s="28"/>
     </row>
-    <row r="13" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1565,7 +1565,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1587,7 +1587,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1609,7 +1609,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1631,7 +1631,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1653,7 +1653,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="G18" s="29"/>
     </row>
-    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1691,7 +1691,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1713,7 +1713,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1735,7 +1735,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1757,7 +1757,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1779,7 +1779,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1801,7 +1801,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1823,7 +1823,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="G26" s="25"/>
     </row>
-    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1861,7 +1861,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>0</v>
@@ -1883,7 +1883,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="G29" s="25"/>
     </row>
-    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1921,7 +1921,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G31" s="17"/>
     </row>
-    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1959,7 +1959,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1981,7 +1981,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>0</v>
@@ -2003,7 +2003,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2019,10 +2019,10 @@
       </c>
       <c r="G35" s="26"/>
     </row>
-    <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" t="s">
         <v>27</v>
@@ -2031,17 +2031,17 @@
         <v>46107</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F36" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>0</v>
@@ -2063,10 +2063,10 @@
         <v>136</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C38" t="s">
         <v>29</v>
@@ -2075,17 +2075,17 @@
         <v>46107</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F38" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G38" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2101,10 +2101,10 @@
       </c>
       <c r="G39" s="26"/>
     </row>
-    <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C40" t="s">
         <v>31</v>
@@ -2113,17 +2113,17 @@
         <v>46107</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F40" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="41" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2145,7 +2145,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2167,7 +2167,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2189,7 +2189,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2211,7 +2211,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2227,7 +2227,7 @@
       </c>
       <c r="G45" s="29"/>
     </row>
-    <row r="46" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>0</v>
@@ -2249,7 +2249,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="47" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>0</v>
@@ -2271,7 +2271,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2293,7 +2293,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2315,7 +2315,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2337,7 +2337,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2359,7 +2359,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="52" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2381,7 +2381,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="53" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2403,7 +2403,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="54" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2425,7 +2425,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="55" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="G55" s="29"/>
     </row>
-    <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2463,7 +2463,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="57" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2485,7 +2485,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="58" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2507,7 +2507,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="59" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2529,7 +2529,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="60" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="G60" s="29"/>
     </row>
-    <row r="61" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2567,7 +2567,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="62" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2589,7 +2589,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="63" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2611,7 +2611,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="64" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="G64" s="29"/>
     </row>
-    <row r="65" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2649,7 +2649,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="66" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2671,7 +2671,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="67" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2693,7 +2693,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2715,7 +2715,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="69" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="G69" s="29"/>
     </row>
-    <row r="70" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2753,7 +2753,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="71" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B71" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2775,7 +2775,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2797,7 +2797,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="73" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B73" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2819,7 +2819,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="74" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2841,7 +2841,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="75" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B75" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G75" s="29"/>
     </row>
-    <row r="76" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2879,7 +2879,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="77" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B77" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2901,7 +2901,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="78" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B78" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2923,7 +2923,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="79" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2945,7 +2945,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="80" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B80" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="G80" s="29"/>
     </row>
-    <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2983,7 +2983,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="82" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B82" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3005,7 +3005,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="83" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B83" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3027,7 +3027,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="84" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B84" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3049,7 +3049,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="85" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B85" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="G85" s="29"/>
     </row>
-    <row r="86" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B86" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3087,7 +3087,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="87" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3109,7 +3109,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="88" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B88" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3131,7 +3131,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="89" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B89" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3153,7 +3153,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="90" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B90" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3175,7 +3175,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="91" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B91" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3197,7 +3197,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="92" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B92" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="G92" s="29"/>
     </row>
-    <row r="93" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B93" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3235,7 +3235,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="94" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B94" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3257,7 +3257,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="95" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B95" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3279,7 +3279,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="96" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B96" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3301,7 +3301,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="97" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B97" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="G97" s="29"/>
     </row>
-    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B98" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3339,7 +3339,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="99" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B99" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3361,7 +3361,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="100" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B100" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3383,7 +3383,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="101" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B101" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3405,7 +3405,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="102" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B102" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="G102" s="29"/>
     </row>
-    <row r="103" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3443,7 +3443,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="104" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B104" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3465,7 +3465,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="105" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B105" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3487,7 +3487,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="106" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B106" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3509,7 +3509,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="107" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B107" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="G107" s="29"/>
     </row>
-    <row r="108" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B108" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3547,7 +3547,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="109" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B109" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3569,7 +3569,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="110" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B110" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3585,7 +3585,7 @@
       </c>
       <c r="G110" s="29"/>
     </row>
-    <row r="111" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B111" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3607,7 +3607,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="112" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B112" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3629,7 +3629,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="113" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B113" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3651,7 +3651,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="114" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B114" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3673,7 +3673,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="115" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B115" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="G115" s="29"/>
     </row>
-    <row r="116" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B116" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3711,7 +3711,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="117" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B117" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3733,7 +3733,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="118" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B118" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="G118" s="29"/>
     </row>
-    <row r="119" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B119" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3771,7 +3771,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="120" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B120" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3793,7 +3793,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="121" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B121" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3815,7 +3815,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="122" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B122" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3837,7 +3837,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="123" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B123" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="G123" s="29"/>
     </row>
-    <row r="124" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B124" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3875,7 +3875,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="125" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B125" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3897,7 +3897,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="126" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B126" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3919,7 +3919,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="127" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B127" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3941,7 +3941,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="128" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B128" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3963,7 +3963,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="129" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B129" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="G129" s="29"/>
     </row>
-    <row r="130" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B130" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -4001,7 +4001,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="131" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B131" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -4023,7 +4023,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="132" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B132" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>

</xml_diff>

<commit_message>
Update project-plan phase 2
</commit_message>
<xml_diff>
--- a/Documentation/project-plan.xlsx
+++ b/Documentation/project-plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanji\Documents\GitHub\IPT6.1-Productivity-Game\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24884F2A-0C21-4041-B639-0A879839CBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF27B85D-8A77-41CA-8CC6-5056F42442BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2820" yWindow="4440" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Idea Planner" sheetId="1" r:id="rId1"/>
@@ -1864,7 +1864,7 @@
     <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" t="s">
         <v>23</v>
@@ -1873,11 +1873,11 @@
         <v>46093</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F28" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" s="11" t="s">
         <v>139</v>
@@ -2104,7 +2104,7 @@
     <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C40" t="s">
         <v>31</v>
@@ -2113,11 +2113,11 @@
         <v>46107</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F40" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="27" t="s">
         <v>136</v>
@@ -2126,7 +2126,7 @@
     <row r="41" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C41" t="s">
         <v>32</v>
@@ -2135,11 +2135,11 @@
         <v>46107</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F41" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G41" s="27" t="s">
         <v>136</v>
@@ -2148,7 +2148,7 @@
     <row r="42" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C42" t="s">
         <v>33</v>
@@ -2157,11 +2157,11 @@
         <v>46107</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F42" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G42" s="27" t="s">
         <v>136</v>
@@ -2170,7 +2170,7 @@
     <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C43" t="s">
         <v>30</v>
@@ -2179,11 +2179,11 @@
         <v>46112</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F43" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G43" s="27" t="s">
         <v>136</v>
@@ -2192,7 +2192,7 @@
     <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C44" t="s">
         <v>34</v>
@@ -2201,11 +2201,11 @@
         <v>46112</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F44" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G44" s="27" t="s">
         <v>136</v>

</xml_diff>

<commit_message>
Update project-plan, phase 2.2, 2.3, 3.1, 3.2, 5.1
</commit_message>
<xml_diff>
--- a/Documentation/project-plan.xlsx
+++ b/Documentation/project-plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanji\Documents\GitHub\IPT6.1-Productivity-Game\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF27B85D-8A77-41CA-8CC6-5056F42442BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{155DAF71-91F2-4C14-BC65-8E1076842942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2820" yWindow="4440" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2044,7 +2044,7 @@
     <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C37" t="s">
         <v>28</v>
@@ -2053,11 +2053,11 @@
         <v>46107</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F37" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" s="27" t="s">
         <v>136</v>
@@ -2066,7 +2066,7 @@
     <row r="38" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C38" t="s">
         <v>29</v>
@@ -2075,11 +2075,11 @@
         <v>46107</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F38" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" s="27" t="s">
         <v>136</v>
@@ -2170,7 +2170,7 @@
     <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C43" t="s">
         <v>30</v>
@@ -2179,11 +2179,11 @@
         <v>46112</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F43" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" s="27" t="s">
         <v>136</v>
@@ -2192,7 +2192,7 @@
     <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C44" t="s">
         <v>34</v>
@@ -2201,11 +2201,11 @@
         <v>46112</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F44" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44" s="27" t="s">
         <v>136</v>
@@ -2230,7 +2230,7 @@
     <row r="46" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C46" t="s">
         <v>42</v>
@@ -2239,11 +2239,11 @@
         <v>46107</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F46" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46" s="27" t="s">
         <v>138</v>
@@ -2252,7 +2252,7 @@
     <row r="47" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C47" t="s">
         <v>141</v>
@@ -2261,11 +2261,11 @@
         <v>46107</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F47" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" s="27" t="s">
         <v>138</v>
@@ -2274,7 +2274,7 @@
     <row r="48" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C48" t="s">
         <v>142</v>
@@ -2283,11 +2283,11 @@
         <v>46112</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F48" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G48" s="27" t="s">
         <v>138</v>
@@ -2296,7 +2296,7 @@
     <row r="49" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C49" t="s">
         <v>143</v>
@@ -2305,11 +2305,11 @@
         <v>46112</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F49" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G49" s="27" t="s">
         <v>138</v>
@@ -2318,7 +2318,7 @@
     <row r="50" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C50" t="s">
         <v>43</v>
@@ -2327,11 +2327,11 @@
         <v>46135</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F50" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G50" s="27" t="s">
         <v>136</v>
@@ -2340,7 +2340,7 @@
     <row r="51" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C51" t="s">
         <v>44</v>
@@ -2349,11 +2349,11 @@
         <v>46135</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F51" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G51" s="27" t="s">
         <v>136</v>
@@ -2362,7 +2362,7 @@
     <row r="52" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C52" t="s">
         <v>45</v>
@@ -2371,11 +2371,11 @@
         <v>46135</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F52" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G52" s="27" t="s">
         <v>136</v>
@@ -2384,7 +2384,7 @@
     <row r="53" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C53" t="s">
         <v>46</v>
@@ -2393,11 +2393,11 @@
         <v>46135</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F53" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G53" s="27" t="s">
         <v>136</v>
@@ -2406,7 +2406,7 @@
     <row r="54" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C54" t="s">
         <v>47</v>
@@ -2415,11 +2415,11 @@
         <v>46111</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F54" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G54" s="27" t="s">
         <v>138</v>
@@ -2444,7 +2444,7 @@
     <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C56" t="s">
         <v>48</v>
@@ -2453,11 +2453,11 @@
         <v>46111</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F56" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G56" s="27" t="s">
         <v>136</v>
@@ -2466,7 +2466,7 @@
     <row r="57" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C57" t="s">
         <v>49</v>
@@ -2475,11 +2475,11 @@
         <v>46111</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F57" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G57" s="27" t="s">
         <v>136</v>
@@ -2488,7 +2488,7 @@
     <row r="58" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C58" t="s">
         <v>50</v>
@@ -2497,11 +2497,11 @@
         <v>46111</v>
       </c>
       <c r="E58" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F58" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G58" s="27" t="s">
         <v>136</v>
@@ -2510,7 +2510,7 @@
     <row r="59" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C59" t="s">
         <v>51</v>
@@ -2519,11 +2519,11 @@
         <v>46111</v>
       </c>
       <c r="E59" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F59" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G59" s="27" t="s">
         <v>136</v>
@@ -2964,7 +2964,7 @@
     <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C81" t="s">
         <v>67</v>
@@ -2973,11 +2973,11 @@
         <v>46116</v>
       </c>
       <c r="E81" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F81" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G81" s="27" t="s">
         <v>136</v>
@@ -2986,7 +2986,7 @@
     <row r="82" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B82" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C82" t="s">
         <v>68</v>
@@ -2995,11 +2995,11 @@
         <v>46116</v>
       </c>
       <c r="E82" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F82" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G82" s="27" t="s">
         <v>138</v>
@@ -3008,7 +3008,7 @@
     <row r="83" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B83" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C83" t="s">
         <v>69</v>
@@ -3017,11 +3017,11 @@
         <v>46116</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F83" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G83" s="27" t="s">
         <v>138</v>
@@ -3030,7 +3030,7 @@
     <row r="84" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B84" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C84" t="s">
         <v>70</v>
@@ -3039,11 +3039,11 @@
         <v>46116</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F84" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G84" s="27" t="s">
         <v>136</v>

</xml_diff>

<commit_message>
Update project-plan update status
</commit_message>
<xml_diff>
--- a/Documentation/project-plan.xlsx
+++ b/Documentation/project-plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ebiru\code\Informatik-2.Jahr\IPT6.1\IPT6.1-Productivity-Game\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanji\Documents\GitHub\IPT6.1-Productivity-Game\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81DA2D8D-5045-4F29-83E3-00D5AB9149D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD307442-94B5-43E5-AB6D-26BCAC9AFC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Idea Planner" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,8 @@
   <definedNames>
     <definedName name="ColumnTitle1">Tasks[[#Headers],[ Task Status Indicator]]</definedName>
     <definedName name="ColumnTitleRegion1..G5.1">'Idea Planner'!$B$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Idea Planner'!$6:$6</definedName>
     <definedName name="PlanDueDate">'Idea Planner'!$E$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Idea Planner'!$6:$6</definedName>
     <definedName name="RowTitleRegion1..E3">'Idea Planner'!$D$2</definedName>
     <definedName name="RowTitleRegion2..G3">'Idea Planner'!$F$2</definedName>
   </definedNames>
@@ -837,26 +837,26 @@
     </xf>
   </cellXfs>
   <cellStyles count="20">
-    <cellStyle name="Calculation" xfId="16" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Berechnung" xfId="16" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Besuchter Hyperlink" xfId="6" builtinId="9" customBuiltin="1"/>
     <cellStyle name="Center aligned" xfId="9" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Comma" xfId="10" builtinId="3" customBuiltin="1"/>
-    <cellStyle name="Comma [0]" xfId="11" builtinId="6" customBuiltin="1"/>
-    <cellStyle name="Currency" xfId="12" builtinId="4" customBuiltin="1"/>
-    <cellStyle name="Currency [0]" xfId="13" builtinId="7" customBuiltin="1"/>
+    <cellStyle name="Dezimal [0]" xfId="11" builtinId="6" customBuiltin="1"/>
     <cellStyle name="Due Date" xfId="18" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Explanatory Text" xfId="7" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
-    <cellStyle name="Per cent" xfId="14" builtinId="5" customBuiltin="1"/>
+    <cellStyle name="Erklärender Text" xfId="7" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Komma" xfId="10" builtinId="3" customBuiltin="1"/>
+    <cellStyle name="Link" xfId="5" builtinId="8" customBuiltin="1"/>
     <cellStyle name="Plan Due Date" xfId="8" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Prozent" xfId="14" builtinId="5" customBuiltin="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0" customBuiltin="1"/>
     <cellStyle name="Status Icon Text" xfId="19" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
     <cellStyle name="Task Indicator" xfId="17" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Überschrift" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Überschrift 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Überschrift 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Überschrift 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Überschrift 4" xfId="15" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Währung" xfId="12" builtinId="4" customBuiltin="1"/>
+    <cellStyle name="Währung [0]" xfId="13" builtinId="7" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="11">
     <dxf>
@@ -1333,23 +1333,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:G132"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.54296875" customWidth="1"/>
+    <col min="1" max="1" width="2.5546875" customWidth="1"/>
     <col min="2" max="2" width="1" customWidth="1"/>
-    <col min="3" max="3" width="42.54296875" customWidth="1"/>
-    <col min="4" max="4" width="18.54296875" customWidth="1"/>
-    <col min="5" max="5" width="22.54296875" customWidth="1"/>
+    <col min="3" max="3" width="42.5546875" customWidth="1"/>
+    <col min="4" max="4" width="18.5546875" customWidth="1"/>
+    <col min="5" max="5" width="22.5546875" customWidth="1"/>
     <col min="6" max="6" width="31" customWidth="1"/>
-    <col min="7" max="7" width="43.453125" customWidth="1"/>
-    <col min="8" max="8" width="2.54296875" customWidth="1"/>
+    <col min="7" max="7" width="43.44140625" customWidth="1"/>
+    <col min="8" max="8" width="2.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
     </row>
-    <row r="2" spans="2:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
@@ -1363,7 +1363,7 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="2:7" ht="33" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:7" ht="33" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="34"/>
       <c r="C3" s="34"/>
       <c r="D3" s="10" t="s">
@@ -1379,7 +1379,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:7" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B4" s="35" t="s">
         <v>3</v>
       </c>
@@ -1391,7 +1391,7 @@
       <c r="F4" s="35"/>
       <c r="G4" s="35"/>
     </row>
-    <row r="5" spans="2:7" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:7" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="36" t="s">
         <v>144</v>
       </c>
@@ -1403,7 +1403,7 @@
       <c r="F5" s="36"/>
       <c r="G5" s="36"/>
     </row>
-    <row r="6" spans="2:7" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:7" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="8" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="G7" s="26"/>
     </row>
-    <row r="8" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1461,7 +1461,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1483,7 +1483,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1505,7 +1505,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1527,7 +1527,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="G12" s="28"/>
     </row>
-    <row r="13" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1565,7 +1565,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1587,7 +1587,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1609,7 +1609,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1631,7 +1631,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1653,7 +1653,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="G18" s="29"/>
     </row>
-    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1691,7 +1691,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1713,7 +1713,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1735,7 +1735,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1757,7 +1757,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1779,7 +1779,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1801,7 +1801,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1823,7 +1823,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="G26" s="25"/>
     </row>
-    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1861,7 +1861,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1883,7 +1883,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="G29" s="25"/>
     </row>
-    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1921,7 +1921,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G31" s="17"/>
     </row>
-    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1959,7 +1959,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1981,7 +1981,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2003,7 +2003,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="G35" s="26"/>
     </row>
-    <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2041,7 +2041,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2063,7 +2063,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2085,7 +2085,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="G39" s="26"/>
     </row>
-    <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2123,7 +2123,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="41" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2145,7 +2145,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2167,7 +2167,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2189,7 +2189,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2211,7 +2211,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2227,7 +2227,7 @@
       </c>
       <c r="G45" s="29"/>
     </row>
-    <row r="46" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2249,7 +2249,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="47" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2271,7 +2271,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2293,7 +2293,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2315,7 +2315,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2337,7 +2337,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2359,7 +2359,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="52" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2381,7 +2381,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="53" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2403,7 +2403,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="54" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2425,7 +2425,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="55" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2441,10 +2441,10 @@
       </c>
       <c r="G55" s="29"/>
     </row>
-    <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C56" t="s">
         <v>48</v>
@@ -2453,20 +2453,20 @@
         <v>46111</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F56" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="57" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C57" t="s">
         <v>49</v>
@@ -2475,20 +2475,20 @@
         <v>46111</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F57" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G57" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="58" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C58" t="s">
         <v>50</v>
@@ -2497,20 +2497,20 @@
         <v>46111</v>
       </c>
       <c r="E58" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F58" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G58" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="59" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C59" t="s">
         <v>51</v>
@@ -2519,17 +2519,17 @@
         <v>46111</v>
       </c>
       <c r="E59" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F59" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G59" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="60" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="G60" s="29"/>
     </row>
-    <row r="61" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2567,7 +2567,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="62" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2589,7 +2589,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="63" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2611,7 +2611,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="64" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2627,10 +2627,10 @@
       </c>
       <c r="G64" s="29"/>
     </row>
-    <row r="65" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C65" t="s">
         <v>55</v>
@@ -2639,20 +2639,20 @@
         <v>46114</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F65" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G65" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="66" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C66" t="s">
         <v>56</v>
@@ -2661,17 +2661,17 @@
         <v>46114</v>
       </c>
       <c r="E66" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F66" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G66" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="67" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2693,10 +2693,10 @@
         <v>138</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C68" t="s">
         <v>146</v>
@@ -2705,17 +2705,17 @@
         <v>46114</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F68" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G68" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="69" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2731,10 +2731,10 @@
       </c>
       <c r="G69" s="29"/>
     </row>
-    <row r="70" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C70" t="s">
         <v>58</v>
@@ -2743,17 +2743,17 @@
         <v>46114</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F70" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G70" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="71" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2775,7 +2775,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2797,7 +2797,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="73" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2819,10 +2819,10 @@
         <v>138</v>
       </c>
     </row>
-    <row r="74" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C74" t="s">
         <v>62</v>
@@ -2831,17 +2831,17 @@
         <v>46114</v>
       </c>
       <c r="E74" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F74" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G74" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="75" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2857,10 +2857,10 @@
       </c>
       <c r="G75" s="29"/>
     </row>
-    <row r="76" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C76" t="s">
         <v>63</v>
@@ -2869,20 +2869,20 @@
         <v>46116</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F76" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G76" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="77" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B77" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C77" t="s">
         <v>64</v>
@@ -2891,17 +2891,17 @@
         <v>46116</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F77" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G77" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="78" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B78" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2923,10 +2923,10 @@
         <v>138</v>
       </c>
     </row>
-    <row r="79" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B79" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C79" t="s">
         <v>66</v>
@@ -2935,17 +2935,17 @@
         <v>46116</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F79" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G79" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="80" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B80" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="G80" s="29"/>
     </row>
-    <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B81" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -2983,7 +2983,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="82" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B82" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -3005,7 +3005,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="83" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B83" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -3027,10 +3027,10 @@
         <v>139</v>
       </c>
     </row>
-    <row r="84" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B84" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C84" t="s">
         <v>70</v>
@@ -3039,17 +3039,17 @@
         <v>46116</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F84" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G84" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="85" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B85" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3065,10 +3065,10 @@
       </c>
       <c r="G85" s="29"/>
     </row>
-    <row r="86" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B86" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C86" t="s">
         <v>72</v>
@@ -3077,20 +3077,20 @@
         <v>46117</v>
       </c>
       <c r="E86" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F86" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G86" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="87" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B87" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C87" t="s">
         <v>73</v>
@@ -3099,20 +3099,20 @@
         <v>46119</v>
       </c>
       <c r="E87" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F87" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G87" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="88" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B88" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C88" t="s">
         <v>74</v>
@@ -3121,20 +3121,20 @@
         <v>46119</v>
       </c>
       <c r="E88" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F88" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G88" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="89" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B89" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C89" t="s">
         <v>75</v>
@@ -3143,20 +3143,20 @@
         <v>46119</v>
       </c>
       <c r="E89" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F89" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G89" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="90" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B90" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C90" t="s">
         <v>76</v>
@@ -3165,20 +3165,20 @@
         <v>46120</v>
       </c>
       <c r="E90" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F90" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G90" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="91" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B91" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C91" t="s">
         <v>77</v>
@@ -3187,17 +3187,17 @@
         <v>46120</v>
       </c>
       <c r="E91" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F91" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G91" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="92" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B92" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3213,10 +3213,10 @@
       </c>
       <c r="G92" s="29"/>
     </row>
-    <row r="93" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B93" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C93" t="s">
         <v>79</v>
@@ -3225,20 +3225,20 @@
         <v>46123</v>
       </c>
       <c r="E93" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F93" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G93" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="94" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B94" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C94" t="s">
         <v>80</v>
@@ -3247,20 +3247,20 @@
         <v>46123</v>
       </c>
       <c r="E94" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F94" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G94" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="95" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B95" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C95" t="s">
         <v>81</v>
@@ -3269,20 +3269,20 @@
         <v>46123</v>
       </c>
       <c r="E95" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F95" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G95" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="96" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B96" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C96" t="s">
         <v>82</v>
@@ -3291,17 +3291,17 @@
         <v>46123</v>
       </c>
       <c r="E96" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F96" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G96" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="97" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B97" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3317,10 +3317,10 @@
       </c>
       <c r="G97" s="29"/>
     </row>
-    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B98" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C98" t="s">
         <v>99</v>
@@ -3329,20 +3329,20 @@
         <v>46123</v>
       </c>
       <c r="E98" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F98" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G98" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="99" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B99" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C99" t="s">
         <v>100</v>
@@ -3351,20 +3351,20 @@
         <v>46125</v>
       </c>
       <c r="E99" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F99" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G99" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="100" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B100" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C100" t="s">
         <v>101</v>
@@ -3373,20 +3373,20 @@
         <v>46125</v>
       </c>
       <c r="E100" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F100" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G100" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="101" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B101" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C101" t="s">
         <v>102</v>
@@ -3395,17 +3395,17 @@
         <v>46125</v>
       </c>
       <c r="E101" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F101" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G101" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="102" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B102" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3421,10 +3421,10 @@
       </c>
       <c r="G102" s="29"/>
     </row>
-    <row r="103" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B103" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C103" t="s">
         <v>104</v>
@@ -3433,20 +3433,20 @@
         <v>46128</v>
       </c>
       <c r="E103" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F103" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G103" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="104" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B104" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C104" t="s">
         <v>105</v>
@@ -3455,20 +3455,20 @@
         <v>46128</v>
       </c>
       <c r="E104" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F104" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G104" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="105" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B105" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C105" t="s">
         <v>106</v>
@@ -3477,20 +3477,20 @@
         <v>46128</v>
       </c>
       <c r="E105" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F105" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G105" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="106" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B106" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C106" t="s">
         <v>107</v>
@@ -3499,17 +3499,17 @@
         <v>46128</v>
       </c>
       <c r="E106" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F106" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G106" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="107" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B107" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3525,10 +3525,10 @@
       </c>
       <c r="G107" s="29"/>
     </row>
-    <row r="108" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B108" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C108" t="s">
         <v>109</v>
@@ -3537,20 +3537,20 @@
         <v>46133</v>
       </c>
       <c r="E108" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F108" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G108" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="109" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B109" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C109" t="s">
         <v>110</v>
@@ -3559,17 +3559,17 @@
         <v>46133</v>
       </c>
       <c r="E109" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F109" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G109" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="110" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B110" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3585,7 +3585,7 @@
       </c>
       <c r="G110" s="29"/>
     </row>
-    <row r="111" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B111" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -3607,10 +3607,10 @@
         <v>138</v>
       </c>
     </row>
-    <row r="112" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B112" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C112" t="s">
         <v>113</v>
@@ -3619,20 +3619,20 @@
         <v>46142</v>
       </c>
       <c r="E112" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F112" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G112" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="113" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B113" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C113" t="s">
         <v>114</v>
@@ -3641,20 +3641,20 @@
         <v>46142</v>
       </c>
       <c r="E113" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F113" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G113" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="114" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B114" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C114" t="s">
         <v>115</v>
@@ -3663,17 +3663,17 @@
         <v>46142</v>
       </c>
       <c r="E114" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F114" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G114" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="115" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B115" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3689,10 +3689,10 @@
       </c>
       <c r="G115" s="29"/>
     </row>
-    <row r="116" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B116" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C116" t="s">
         <v>117</v>
@@ -3701,20 +3701,20 @@
         <v>46156</v>
       </c>
       <c r="E116" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F116" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G116" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="117" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B117" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C117" t="s">
         <v>118</v>
@@ -3723,17 +3723,17 @@
         <v>46156</v>
       </c>
       <c r="E117" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F117" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G117" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="118" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B118" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3749,10 +3749,10 @@
       </c>
       <c r="G118" s="29"/>
     </row>
-    <row r="119" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B119" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C119" t="s">
         <v>120</v>
@@ -3761,17 +3761,17 @@
         <v>46163</v>
       </c>
       <c r="E119" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F119" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G119" s="27" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="120" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B120" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -3793,10 +3793,10 @@
         <v>138</v>
       </c>
     </row>
-    <row r="121" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B121" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C121" t="s">
         <v>122</v>
@@ -3805,20 +3805,20 @@
         <v>46170</v>
       </c>
       <c r="E121" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F121" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G121" s="27" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="122" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B122" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C122" t="s">
         <v>123</v>
@@ -3827,17 +3827,17 @@
         <v>46170</v>
       </c>
       <c r="E122" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F122" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G122" s="27" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="123" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B123" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3853,10 +3853,10 @@
       </c>
       <c r="G123" s="29"/>
     </row>
-    <row r="124" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B124" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C124" t="s">
         <v>125</v>
@@ -3865,20 +3865,20 @@
         <v>46177</v>
       </c>
       <c r="E124" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F124" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G124" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="125" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B125" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C125" t="s">
         <v>126</v>
@@ -3887,17 +3887,17 @@
         <v>46177</v>
       </c>
       <c r="E125" s="13" t="s">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="F125" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G125" s="27" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="126" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B126" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -3919,10 +3919,10 @@
         <v>138</v>
       </c>
     </row>
-    <row r="127" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B127" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C127" t="s">
         <v>128</v>
@@ -3931,20 +3931,20 @@
         <v>46177</v>
       </c>
       <c r="E127" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F127" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G127" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="128" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B128" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C128" t="s">
         <v>129</v>
@@ -3953,17 +3953,17 @@
         <v>46177</v>
       </c>
       <c r="E128" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F128" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G128" s="27" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="129" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B129" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="G129" s="29"/>
     </row>
-    <row r="130" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B130" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -4001,10 +4001,10 @@
         <v>138</v>
       </c>
     </row>
-    <row r="131" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B131" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C131" t="s">
         <v>145</v>
@@ -4013,20 +4013,20 @@
         <v>46185</v>
       </c>
       <c r="E131" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F131" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G131" s="27" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="132" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B132" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C132" t="s">
         <v>132</v>
@@ -4035,11 +4035,11 @@
         <v>46185</v>
       </c>
       <c r="E132" s="13" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="F132" s="11">
         <f ca="1">IFERROR(IF(ISBLANK(Tasks[[#This Row],[Due Date]]),"",IF(Tasks[[#This Row],[Done?]]="Yes",1,IF(OR(Tasks[[#This Row],[Due Date]]&gt;PlanDueDate,Tasks[[#This Row],[Done?]]="No"),-1,IF(OR(OR(Tasks[[#This Row],[Due Date]]=TODAY(),Tasks[[#This Row],[Due Date]]=PlanDueDate),Tasks[[#This Row],[Done?]]="Pending"),0,"")))),"")</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G132" s="27" t="s">
         <v>136</v>

</xml_diff>